<commit_message>
Phase 1: re-anchor physics — demand base to gross generation (37.09 TWh), hydro to measured 11.47 TWh, gas deliverability to 89.27 TWh_th; backcast reproduces observed 2024 gas generation within 4%
</commit_message>
<xml_diff>
--- a/data/gas/processed/gas_to_power_reconciliation_2025H1.xlsx
+++ b/data/gas/processed/gas_to_power_reconciliation_2025H1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Desktop\MSc\AUST\Thesis\thesis-repo\thesis-code\data\gas\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5E73703-E76D-499C-BFC0-D4CF7C6C378E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{096C1308-F07D-4BE9-A68B-4FDA2650C42E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11520" yWindow="0" windowWidth="11520" windowHeight="12360" xr2:uid="{41EBFF8F-819B-4B9E-BE44-3162811BFB4A}"/>
+    <workbookView xWindow="10752" yWindow="0" windowWidth="11724" windowHeight="12228" xr2:uid="{41EBFF8F-819B-4B9E-BE44-3162811BFB4A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,14 +25,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t>Period</t>
   </si>
   <si>
-    <t>2025 (Q1-Q3)</t>
-  </si>
-  <si>
     <t>gas_to_power_mmscf</t>
   </si>
   <si>
@@ -58,6 +55,12 @@
   </si>
   <si>
     <t>heating_value_btu_per_scf(HHV)</t>
+  </si>
+  <si>
+    <t>gas_generation TWh_e</t>
+  </si>
+  <si>
+    <t>gas_to_power TWh_e</t>
   </si>
 </sst>
 </file>
@@ -432,7 +435,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D1DE5C9-8DC7-4ED9-BD7C-48F6B5B41F70}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.88671875" bestFit="1" customWidth="1"/>
@@ -449,30 +452,30 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
+      <c r="A2" s="2">
+        <v>2025</v>
       </c>
       <c r="B2" s="3">
         <v>153878.72</v>
@@ -496,12 +499,38 @@
         <v>69333307160000</v>
       </c>
       <c r="H2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H3" t="s">
-        <v>9</v>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E7">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E8">
+        <v>0.28999999999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E9">
+        <v>0.31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>